<commit_message>
Validacion de documentos fechas telefonos y perfiles
</commit_message>
<xml_diff>
--- a/parametros.xlsx
+++ b/parametros.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onesofttek-my.sharepoint.com/personal/mabel_acevedo_softtek_com/Documents/Documents/proyecto_acevedo/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{C1443F39-4474-4A47-A7BD-35A0B96D73B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0289F368-2F12-4EFD-97AD-12AC3D86A4A4}"/>
+  <xr:revisionPtr revIDLastSave="173" documentId="8_{C1443F39-4474-4A47-A7BD-35A0B96D73B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{332D6089-A91F-4F76-961F-A737C4170C94}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{9698D67A-5D04-41E4-8055-857222EE1972}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{9698D67A-5D04-41E4-8055-857222EE1972}"/>
   </bookViews>
   <sheets>
     <sheet name="Parametros" sheetId="1" r:id="rId1"/>
@@ -43,13 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
-  <si>
-    <t>clave</t>
-  </si>
-  <si>
-    <t>valor</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="66">
   <si>
     <t>dominio_correo</t>
   </si>
@@ -97,6 +91,221 @@
   </si>
   <si>
     <t>campos_requeridos</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">                 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nombre</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">     </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>codigo</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">                 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>area</t>
+    </r>
+  </si>
+  <si>
+    <t>CC-1040</t>
+  </si>
+  <si>
+    <t>CC-1050</t>
+  </si>
+  <si>
+    <t>CC-2010</t>
+  </si>
+  <si>
+    <t>CC-3010</t>
+  </si>
+  <si>
+    <t>Desarrollo de software</t>
+  </si>
+  <si>
+    <t>Soporte operación</t>
+  </si>
+  <si>
+    <t>Consultoria funcional</t>
+  </si>
+  <si>
+    <t>Administracion finanzas</t>
+  </si>
+  <si>
+    <t>Tecnologia</t>
+  </si>
+  <si>
+    <t>Consultoria</t>
+  </si>
+  <si>
+    <t>Administracion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     codigo_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     nombre_cargo</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">   </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>nivel</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">                </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>area</t>
+    </r>
+  </si>
+  <si>
+    <t>ANL-01</t>
+  </si>
+  <si>
+    <t>ANL-02</t>
+  </si>
+  <si>
+    <t>DES-01</t>
+  </si>
+  <si>
+    <t>CON-01</t>
+  </si>
+  <si>
+    <t>ADM-01</t>
+  </si>
+  <si>
+    <t>GER-01</t>
+  </si>
+  <si>
+    <t>Analista junior</t>
+  </si>
+  <si>
+    <t>Analista senior</t>
+  </si>
+  <si>
+    <t>Desarrollador</t>
+  </si>
+  <si>
+    <t>Consultor funcional</t>
+  </si>
+  <si>
+    <t>Auxiliar administrativo</t>
+  </si>
+  <si>
+    <t>Gerente area</t>
+  </si>
+  <si>
+    <t>requiere_aprobacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">             perfil_sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">              area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   codigo_cargo</t>
+  </si>
+  <si>
+    <t>Perf_analista_bas</t>
+  </si>
+  <si>
+    <t>Perf_analista_avz</t>
+  </si>
+  <si>
+    <t>Perfil_desarrollo</t>
+  </si>
+  <si>
+    <t>Perfil_consultor</t>
+  </si>
+  <si>
+    <t>Perf_admin_bas</t>
+  </si>
+  <si>
+    <t>Perf_gerencial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">               si</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      clave</t>
+  </si>
+  <si>
+    <t>formato_fecha_salida</t>
+  </si>
+  <si>
+    <t>AAAA-MM-DD</t>
+  </si>
+  <si>
+    <t>dias_maximo_futuro</t>
+  </si>
+  <si>
+    <t>longitud_telefono</t>
+  </si>
+  <si>
+    <t>nivel_log_minimo</t>
+  </si>
+  <si>
+    <t>INFO</t>
   </si>
 </sst>
 </file>
@@ -158,6 +367,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -477,43 +690,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A4472651-8DC3-41E7-970A-551CF350B835}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
     <col min="2" max="2" width="16.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
+      <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -523,27 +768,297 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A7FDAC6-8787-478D-B98A-9E46FE65A73E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21.140625" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{512BC253-D02A-4AB8-9C13-4F0C69AE0344}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="23.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6170F061-5A01-49AE-BC86-F5BA98CA095D}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -553,47 +1068,48 @@
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="18.5703125" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="91.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>